<commit_message>
data(gold-gears): G08-P3-B6 verify sora and visual qa
</commit_message>
<xml_diff>
--- a/config/gold-and-gears/data/GoldAndGearsProgression.xlsx
+++ b/config/gold-and-gears/data/GoldAndGearsProgression.xlsx
@@ -10435,7 +10435,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="72" customHeight="1">
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="8" t="n">
         <v>33</v>
@@ -12949,7 +12949,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="9" t="n"/>
       <c r="B9" s="9" t="n">
         <v>2</v>
@@ -13734,7 +13734,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="72" customHeight="1">
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="8" t="n">
         <v>7</v>
@@ -13891,7 +13891,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="72" customHeight="1">
       <c r="A15" s="9" t="n"/>
       <c r="B15" s="9" t="n">
         <v>8</v>
@@ -14052,7 +14052,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="72" customHeight="1">
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="8" t="n">
         <v>9</v>
@@ -14209,7 +14209,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="72" customHeight="1">
       <c r="A17" s="9" t="n"/>
       <c r="B17" s="9" t="n">
         <v>10</v>
@@ -14370,7 +14370,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="72" customHeight="1">
       <c r="A18" s="8" t="n"/>
       <c r="B18" s="8" t="n">
         <v>11</v>
@@ -14527,7 +14527,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="72" customHeight="1">
       <c r="A19" s="9" t="n"/>
       <c r="B19" s="9" t="n">
         <v>12</v>

</xml_diff>